<commit_message>
fixed subject and message line
</commit_message>
<xml_diff>
--- a/arrays.xlsx
+++ b/arrays.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="510">
   <si>
     <t>Message 1 of 126</t>
   </si>
@@ -46,9 +46,6 @@
     <t>To: Laura Lowe (First Viewed: 06/07/2022 at 03:19 PM)</t>
   </si>
   <si>
-    <t>Subject: RE: Test Message</t>
-  </si>
-  <si>
     <t>ok my account is set up and they refunded your card.</t>
   </si>
   <si>
@@ -76,9 +73,6 @@
     <t>To: John Lowe (First Viewed: 06/08/2022 at 01:16 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Real Estate Agent</t>
-  </si>
-  <si>
     <t>I will look at the schedule and get back to you.</t>
   </si>
   <si>
@@ -91,9 +85,6 @@
     <t>To: Laura Lowe (First Viewed: 06/08/2022 at 03:21 PM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: Real Estate Agent</t>
-  </si>
-  <si>
     <t>ok thanks</t>
   </si>
   <si>
@@ -106,9 +97,6 @@
     <t>To: John Lowe (First Viewed: 06/08/2022 at 03:24 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Re: Real Estate Agent</t>
-  </si>
-  <si>
     <t>Laura</t>
   </si>
   <si>
@@ -136,9 +124,6 @@
     <t>To: John Lowe (First Viewed: 06/08/2022 at 04:20 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: John's football conditioning tonight</t>
-  </si>
-  <si>
     <t>He is taking this week off from football practice.</t>
   </si>
   <si>
@@ -163,9 +148,6 @@
     <t>To: Laura Lowe (First Viewed: 06/08/2022 at 04:35 PM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: John's football conditioning tonight</t>
-  </si>
-  <si>
     <t>Message 11 of 126</t>
   </si>
   <si>
@@ -184,9 +166,6 @@
     <t>To: John Lowe (First Viewed: 06/08/2022 at 04:38 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Re: John's football conditioning tonight</t>
-  </si>
-  <si>
     <t>I have the phone app and it sends notifications.</t>
   </si>
   <si>
@@ -199,10 +178,7 @@
     <t>To: Laura Lowe (First Viewed: 06/09/2022 at 11:44 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Test Message</t>
-  </si>
-  <si>
-    <t>I signed up for Zelle so you can pay me for half of the subscription through that if it is easier for you. Just use my cell number.</t>
+    <t>I signed up for Zelle so you can pay me for half of the subscription through that if it is easier fo</t>
   </si>
   <si>
     <t>Message 14 of 126</t>
@@ -229,6 +205,9 @@
     <t>Subject: Clothes and Shoes</t>
   </si>
   <si>
+    <t>Let me know if you need their sizes.</t>
+  </si>
+  <si>
     <t>Message 16 of 126</t>
   </si>
   <si>
@@ -238,9 +217,6 @@
     <t>To: Laura Lowe (First Viewed: 06/11/2022 at 07:45 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Clothes and Shoes</t>
-  </si>
-  <si>
     <t>I will most likely need stuff thru the summer schedule.</t>
   </si>
   <si>
@@ -253,7 +229,7 @@
     <t>To: John Lowe (First Viewed: 06/11/2022 at 07:48 AM)</t>
   </si>
   <si>
-    <t>I’m happy to send clothes but Target and Amazon have everything they need so why do you need me to send clothes all summer?</t>
+    <t>I’m happy to send clothes but Target and Amazon have everything they need so why do you need me to s</t>
   </si>
   <si>
     <t>Message 18 of 126</t>
@@ -307,9 +283,6 @@
     <t>To: Laura Lowe (First Viewed: 06/12/2022 at 08:57 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Football Training</t>
-  </si>
-  <si>
     <t>Yes he will go Wednesday but probably not Thursday</t>
   </si>
   <si>
@@ -325,7 +298,7 @@
     <t>Subject: John’s practice tonight</t>
   </si>
   <si>
-    <t>leaving pets or children in unattended vehicles. Anyone overcome by heat should be moved to a cool and shaded location.</t>
+    <t>leaving pets or children in unattended vehicles. Anyone overcome by heat should be moved to a cool a</t>
   </si>
   <si>
     <t>Message 23 of 126</t>
@@ -334,9 +307,6 @@
     <t>Sent: 06/13/2022 at 09:16 AM</t>
   </si>
   <si>
-    <t>Subject: Re: Kids Sizes</t>
-  </si>
-  <si>
     <t>Message 24 of 126</t>
   </si>
   <si>
@@ -346,9 +316,6 @@
     <t>To: John Lowe (First Viewed: 06/13/2022 at 09:21 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: John’s practice tonight</t>
-  </si>
-  <si>
     <t>Message 25 of 126</t>
   </si>
   <si>
@@ -361,7 +328,7 @@
     <t>Subject: Colorado Trip</t>
   </si>
   <si>
-    <t>We are flying direct into Albuquerque and renting a car and driving to Durango because of the complications of connecting flights and layovers.</t>
+    <t>We are flying direct into Albuquerque and renting a car and driving to Durango because of the compli</t>
   </si>
   <si>
     <t>Message 26 of 126</t>
@@ -373,9 +340,6 @@
     <t>To: Laura Lowe (First Viewed: 06/13/2022 at 11:22 AM)</t>
   </si>
   <si>
-    <t>Subject: RE: Colorado Trip</t>
-  </si>
-  <si>
     <t>Message 27 of 126</t>
   </si>
   <si>
@@ -394,9 +358,6 @@
     <t>Sent: 06/13/2022 at 11:24 AM</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Colorado Trip</t>
-  </si>
-  <si>
     <t>Jason’s contact information</t>
   </si>
   <si>
@@ -439,9 +400,6 @@
     <t>To: Laura Lowe (First Viewed: 06/15/2022 at 09:48 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Pick up today</t>
-  </si>
-  <si>
     <t>you are supposed to drop them off at 6pm</t>
   </si>
   <si>
@@ -493,9 +451,6 @@
     <t>To: Laura Lowe (First Viewed: 06/15/2022 at 04:56 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Drop off 5:55pm</t>
-  </si>
-  <si>
     <t>Message 37 of 126</t>
   </si>
   <si>
@@ -520,9 +475,6 @@
     <t>To: Laura Lowe (First Viewed: 06/16/2022 at 10:10 AM)</t>
   </si>
   <si>
-    <t>Subject: RE: Melatonin</t>
-  </si>
-  <si>
     <t>ok. He went right to sleep last night. I can get some at Publix if he needs it.</t>
   </si>
   <si>
@@ -547,10 +499,7 @@
     <t>To: John Lowe (First Viewed: 06/16/2022 at 12:41 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: House Photographer</t>
-  </si>
-  <si>
-    <t>I will not be home tomorrow but for a brief period. The next day I have available is Monday or another day next week.</t>
+    <t>I will not be home tomorrow but for a brief period. The next day I have available is Monday or anoth</t>
   </si>
   <si>
     <t>Message 41 of 126</t>
@@ -586,9 +535,6 @@
     <t>To: Laura Lowe (First Viewed: 06/17/2022 at 07:38 AM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: House Photographer</t>
-  </si>
-  <si>
     <t>I will have then plan on that time.</t>
   </si>
   <si>
@@ -616,9 +562,6 @@
     <t>To: John Lowe (First Viewed: 06/17/2022 at 11:26 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Lori's notes for listing the house</t>
-  </si>
-  <si>
     <t>Is the open house scheduled for the dates she listed?</t>
   </si>
   <si>
@@ -655,7 +598,7 @@
     <t>To: John Lowe (First Viewed: 06/17/2022 at 04:00 PM)</t>
   </si>
   <si>
-    <t>My work schedule comes out Sunday night so I will look at next weekend for you to pack up the office.</t>
+    <t>My work schedule comes out Sunday night so I will look at next weekend for you to pack up the office</t>
   </si>
   <si>
     <t>Message 49 of 126</t>
@@ -667,10 +610,7 @@
     <t>To: Laura Lowe (First Viewed: 06/17/2022 at 07:09 PM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: Lori's notes for listing the house</t>
-  </si>
-  <si>
-    <t>The blower is gas powered. Brandon has an electric one and I think Clay might as well. Those would be much easier for you to use.</t>
+    <t>The blower is gas powered. Brandon has an electric one and I think Clay might as well. Those would b</t>
   </si>
   <si>
     <t>Message 50 of 126</t>
@@ -682,9 +622,6 @@
     <t>To: John Lowe (First Viewed: 06/17/2022 at 07:33 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Re: Lori's notes for listing the house</t>
-  </si>
-  <si>
     <t>Ms Leonard so she is a better person to get this information from.</t>
   </si>
   <si>
@@ -715,9 +652,6 @@
     <t>To: John Lowe (First Viewed: 06/18/2022 at 09:11 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Re: House Photographer</t>
-  </si>
-  <si>
     <t>11 am works on Monday. I’ll have everything ready for him.</t>
   </si>
   <si>
@@ -730,9 +664,6 @@
     <t>To: Laura Lowe (First Viewed: 06/18/2022 at 06:15 PM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: RE: Re: House Photographer</t>
-  </si>
-  <si>
     <t>Message 55 of 126</t>
   </si>
   <si>
@@ -745,7 +676,7 @@
     <t>Subject: Football training</t>
   </si>
   <si>
-    <t>Is John glimt to football training Monday night?</t>
+    <t>Wednesday and Thursday are going to be 100 degrees.</t>
   </si>
   <si>
     <t>Message 56 of 126</t>
@@ -757,9 +688,6 @@
     <t>To: John Lowe (First Viewed: 06/18/2022 at 06:17 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Football training</t>
-  </si>
-  <si>
     <t>Going not glimt</t>
   </si>
   <si>
@@ -772,7 +700,7 @@
     <t>To: Laura Lowe (First Viewed: 06/18/2022 at 07:11 PM)</t>
   </si>
   <si>
-    <t>They have been cancelling the practice. We will play it by ear but if it is that hot I doubt they even have it.</t>
+    <t>They have been cancelling the practice. We will play it by ear but if it is that hot I doubt they ev</t>
   </si>
   <si>
     <t>Message 58 of 126</t>
@@ -787,7 +715,7 @@
     <t>Subject: Noah Speech Therapy</t>
   </si>
   <si>
-    <t>Noah has speech therapy tomorrow at 12:15 at Smyrna Prep. I am attaching Michelle’s number if you need to make any changes.</t>
+    <t>Noah has speech therapy tomorrow at 12:15 at Smyrna Prep. I am attaching Michelle’s number if you ne</t>
   </si>
   <si>
     <t>Message 59 of 126</t>
@@ -799,9 +727,6 @@
     <t>To: Laura Lowe (First Viewed: 06/19/2022 at 01:48 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Noah Speech Therapy</t>
-  </si>
-  <si>
     <t>Ok thanks</t>
   </si>
   <si>
@@ -850,9 +775,6 @@
     <t>To: Laura Lowe (First Viewed: 06/20/2022 at 10:12 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Office Pack Up</t>
-  </si>
-  <si>
     <t>cancels I will let you know.</t>
   </si>
   <si>
@@ -901,7 +823,7 @@
     <t>To: John Lowe (First Viewed: 06/20/2022 at 12:09 PM)</t>
   </si>
   <si>
-    <t>We moved a few things around to optimize photo quality. The backyard needs TLC but overall he said the photos turned out great.</t>
+    <t>We moved a few things around to optimize photo quality. The backyard needs TLC but overall he said t</t>
   </si>
   <si>
     <t>Message 68 of 126</t>
@@ -1042,9 +964,6 @@
     <t>To: Laura Lowe (First Viewed: 06/23/2022 at 08:12 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: FaceTime</t>
-  </si>
-  <si>
     <t>Message 80 of 126</t>
   </si>
   <si>
@@ -1057,7 +976,7 @@
     <t>Subject: John Jr Orthodontist</t>
   </si>
   <si>
-    <t>John has an orthodontist appt on Monday July 11th at 10am with Dr Cohen. He is going to evaluate John for phase 2 braces.</t>
+    <t>John has an orthodontist appt on Monday July 11th at 10am with Dr Cohen. He is going to evaluate Joh</t>
   </si>
   <si>
     <t>Message 81 of 126</t>
@@ -1069,9 +988,6 @@
     <t>To: Laura Lowe (First Viewed: 06/23/2022 at 09:34 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: John Jr Orthodontist</t>
-  </si>
-  <si>
     <t>I will see if that works for me. If not I will reschedule it.</t>
   </si>
   <si>
@@ -1084,7 +1000,7 @@
     <t>To: John Lowe (First Viewed: 06/23/2022 at 09:38 AM)</t>
   </si>
   <si>
-    <t>Please read the parenting plan. I am allowed to take John to the doctor during my parenting time and provide all of the information to you.</t>
+    <t>Please read the parenting plan. I am allowed to take John to the doctor during my parenting time and</t>
   </si>
   <si>
     <t>Message 83 of 126</t>
@@ -1096,9 +1012,6 @@
     <t>To: Laura Lowe (First Viewed: 06/23/2022 at 09:55 AM)</t>
   </si>
   <si>
-    <t>Subject: RE: Re: John Jr Orthodontist</t>
-  </si>
-  <si>
     <t>without my consent.</t>
   </si>
   <si>
@@ -1111,10 +1024,7 @@
     <t>To: John Lowe (First Viewed: 06/23/2022 at 10:00 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: RE: Re: John Jr Orthodontist</t>
-  </si>
-  <si>
-    <t>I will get clarification from my counsel. The Medical Appt Section does not specify “sick or injured”. It says “medical appointments”.</t>
+    <t>I will get clarification from my counsel. The Medical Appt Section does not specify “sick or injured</t>
   </si>
   <si>
     <t>Message 85 of 126</t>
@@ -1153,9 +1063,6 @@
     <t>To: John Lowe (First Viewed: 06/23/2022 at 05:35 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Football conditioning</t>
-  </si>
-  <si>
     <t>Message 88 of 126</t>
   </si>
   <si>
@@ -1168,6 +1075,9 @@
     <t>Subject: Noah off the high dive</t>
   </si>
   <si>
+    <t>See the attached videos of Noah going off the high dive for the first time and John doing a flip off</t>
+  </si>
+  <si>
     <t>Message 89 of 126</t>
   </si>
   <si>
@@ -1177,9 +1087,6 @@
     <t>To: John Lowe (First Viewed: 06/24/2022 at 02:44 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Noah off the high dive</t>
-  </si>
-  <si>
     <t>Awesome thank you</t>
   </si>
   <si>
@@ -1192,7 +1099,7 @@
     <t>To: John Lowe (First Viewed: 06/25/2022 at 08:34 AM)</t>
   </si>
   <si>
-    <t>You are here at the house right now. Saturday, June 25th. You are supposed to be here Sunday June 26th.</t>
+    <t>You are here at the house right now. Saturday, June 25th. You are supposed to be here Sunday June 26</t>
   </si>
   <si>
     <t>Message 91 of 126</t>
@@ -1204,7 +1111,7 @@
     <t>To: John Lowe (First Viewed: 06/25/2022 at 08:35 AM)</t>
   </si>
   <si>
-    <t>I have to be at work this morning. You need to come back tomorrow morning when you are scheduled to be here.</t>
+    <t xml:space="preserve">I have to be at work this morning. You need to come back tomorrow morning when you are scheduled to </t>
   </si>
   <si>
     <t>Message 92 of 126</t>
@@ -1273,9 +1180,6 @@
     <t>To: Laura Lowe (First Viewed: 06/26/2022 at 07:21 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Football Training Monday</t>
-  </si>
-  <si>
     <t>We are planning on going. I will let you know.</t>
   </si>
   <si>
@@ -1306,7 +1210,7 @@
     <t>Subject: Noah</t>
   </si>
   <si>
-    <t>Noah is running a fever this morning so he is going to stay home from school. He says he feels fine otherwise.</t>
+    <t xml:space="preserve">Noah is running a fever this morning so he is going to stay home from school. He says he feels fine </t>
   </si>
   <si>
     <t>Message 100 of 126</t>
@@ -1318,9 +1222,6 @@
     <t>To: John Lowe (First Viewed: 06/27/2022 at 07:35 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Noah</t>
-  </si>
-  <si>
     <t>Please let Michelle Phillips and the school know. He is scheduled for speech at 12:15.</t>
   </si>
   <si>
@@ -1348,9 +1249,6 @@
     <t>To: John Lowe (First Viewed: 06/27/2022 at 08:46 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Speech therapy</t>
-  </si>
-  <si>
     <t>Thank you. I will coordinate with Michelle.</t>
   </si>
   <si>
@@ -1366,7 +1264,7 @@
     <t>Subject: New Address</t>
   </si>
   <si>
-    <t>John and Noah said you are moving to a new address/house. Can you please tell me where your moving? The address?</t>
+    <t xml:space="preserve">John and Noah said you are moving to a new address/house. Can you please tell me where your moving? </t>
   </si>
   <si>
     <t>Message 104 of 126</t>
@@ -1378,9 +1276,6 @@
     <t>To: Laura Lowe (First Viewed: 06/28/2022 at 02:51 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: New Address</t>
-  </si>
-  <si>
     <t>We are in the process of moving. The new address will be 1010 ridgecrest drive smyrna.</t>
   </si>
   <si>
@@ -1393,7 +1288,7 @@
     <t>To: John Lowe (First Viewed: 06/28/2022 at 02:52 PM)</t>
   </si>
   <si>
-    <t>John and Noah said you were spending the night at the new house last night. Did you spend the night or when will you be officially in the house?</t>
+    <t xml:space="preserve">John and Noah said you were spending the night at the new house last night. Did you spend the night </t>
   </si>
   <si>
     <t>Message 106 of 126</t>
@@ -1441,9 +1336,6 @@
     <t>To: John Lowe (First Viewed: 06/29/2022 at 10:12 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Amanda Jones’ email</t>
-  </si>
-  <si>
     <t>curriculum and evaluate and re-evaluate. I think we should see how Amanda’s suggestion fits in.</t>
   </si>
   <si>
@@ -1456,9 +1348,6 @@
     <t>To: John Lowe (First Viewed: 06/29/2022 at 11:36 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Tax info</t>
-  </si>
-  <si>
     <t>I sent my 1099 to your email because I can’t get it to attach here. Send me the amended return.</t>
   </si>
   <si>
@@ -1534,9 +1423,6 @@
     <t>To: John Lowe (First Viewed: 06/29/2022 at 05:16 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Practice</t>
-  </si>
-  <si>
     <t>I am at work and won’t be there.</t>
   </si>
   <si>
@@ -1549,9 +1435,6 @@
     <t>To: John Lowe (First Viewed: 06/29/2022 at 05:17 PM)</t>
   </si>
   <si>
-    <t>Subject: Re: Lawnmower</t>
-  </si>
-  <si>
     <t>Let’s settle it with personal property list.</t>
   </si>
   <si>
@@ -1582,7 +1465,7 @@
     <t>To: John Lowe (First Viewed: 06/29/2022 at 06:49 PM)</t>
   </si>
   <si>
-    <t>You have taken many items, furniture from the house without question or opposition. The rest is on the personal property inventory list</t>
+    <t>You have taken many items, furniture from the house without question or opposition. The rest is on t</t>
   </si>
   <si>
     <t>Message 121 of 126</t>
@@ -1609,9 +1492,6 @@
     <t>To: John Lowe (First Viewed: 06/30/2022 at 07:48 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Carlton Haggard</t>
-  </si>
-  <si>
     <t>Message 123 of 126</t>
   </si>
   <si>
@@ -1639,7 +1519,7 @@
     <t>Subject: Office Pack June 26th</t>
   </si>
   <si>
-    <t>I was not aware you were taking marital furniture. The Restoration Hardware desk. I was not informed or asked.</t>
+    <t>I was not aware you were taking marital furniture. The Restoration Hardware desk. I was not informed</t>
   </si>
   <si>
     <t>Message 125 of 126</t>
@@ -1651,9 +1531,6 @@
     <t>To: Laura Lowe (First Viewed: 07/01/2022 at 08:32 AM)</t>
   </si>
   <si>
-    <t>Subject: RE: John Jr Counseling</t>
-  </si>
-  <si>
     <t>wasn't sure if you would do Thursdays.</t>
   </si>
   <si>
@@ -1666,10 +1543,7 @@
     <t>To: John Lowe (First Viewed: 07/01/2022 at 08:42 AM)</t>
   </si>
   <si>
-    <t>Subject: Re: Office Pack June 26th</t>
-  </si>
-  <si>
-    <t>Lori’s notes and your message attached. You were not supposed to move marital furniture, the RH desk out of the house.</t>
+    <t>Lori’s notes and your message attached. You were not supposed to move marital furniture, the RH desk</t>
   </si>
 </sst>
 </file>
@@ -2038,2484 +1912,2490 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
         <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
         <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
         <v>32</v>
-      </c>
-      <c r="B7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
         <v>40</v>
-      </c>
-      <c r="F9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="F12" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s">
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>62</v>
+      </c>
+      <c r="F15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F17" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="F18" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F20" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F21" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="E23" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C24" t="s">
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="E24" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="F24" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="C25" t="s">
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="E25" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="E26" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="F26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="E27" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="F27" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
         <v>2</v>
       </c>
       <c r="D28" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="E28" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="B29" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
       </c>
       <c r="D29" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="E29" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="F29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="B30" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
         <v>8</v>
       </c>
       <c r="D30" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="E30" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="F30" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="C31" t="s">
         <v>2</v>
       </c>
       <c r="D31" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E31" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F31" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="B32" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="C32" t="s">
         <v>8</v>
       </c>
       <c r="D32" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="E32" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="F32" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="C33" t="s">
         <v>2</v>
       </c>
       <c r="D33" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="F33" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="B34" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="C34" t="s">
         <v>8</v>
       </c>
       <c r="D34" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="E34" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="F34" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B35" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C35" t="s">
         <v>2</v>
       </c>
       <c r="D35" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="E35" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="F35" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="B36" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="C36" t="s">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="E36" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="F36" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="B37" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="C37" t="s">
         <v>2</v>
       </c>
       <c r="D37" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="E37" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="F37" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="B38" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="C38" t="s">
         <v>8</v>
       </c>
       <c r="D38" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="E38" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="F38" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="B39" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="C39" t="s">
         <v>8</v>
       </c>
       <c r="D39" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="E39" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="F39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="B40" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="C40" t="s">
         <v>2</v>
       </c>
       <c r="D40" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="E40" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="F40" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
       <c r="B41" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
         <v>8</v>
       </c>
       <c r="D41" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="E41" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="F41" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="B42" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="C42" t="s">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>185</v>
+        <v>168</v>
       </c>
       <c r="E42" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="F42" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" t="s">
-        <v>187</v>
+        <v>170</v>
       </c>
       <c r="B43" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
       <c r="C43" t="s">
         <v>8</v>
       </c>
       <c r="D43" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="E43" t="s">
-        <v>190</v>
+        <v>157</v>
       </c>
       <c r="F43" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="B44" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="C44" t="s">
         <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="E44" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="F44" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B45" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="C45" t="s">
         <v>2</v>
       </c>
       <c r="D45" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="E45" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="F45" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="B46" t="s">
-        <v>203</v>
+        <v>184</v>
       </c>
       <c r="C46" t="s">
         <v>8</v>
       </c>
       <c r="D46" t="s">
-        <v>204</v>
+        <v>185</v>
       </c>
       <c r="E46" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="F46" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" t="s">
-        <v>206</v>
+        <v>187</v>
       </c>
       <c r="B47" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="C47" t="s">
         <v>2</v>
       </c>
       <c r="D47" t="s">
-        <v>208</v>
+        <v>189</v>
       </c>
       <c r="E47" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="F47" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" spans="1:6">
       <c r="A48" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
       <c r="B48" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
         <v>2</v>
       </c>
       <c r="D48" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E48" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="F48" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="B49" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
       <c r="C49" t="s">
         <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="E49" t="s">
-        <v>217</v>
+        <v>177</v>
       </c>
       <c r="F49" t="s">
-        <v>218</v>
+        <v>198</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" t="s">
-        <v>219</v>
+        <v>199</v>
       </c>
       <c r="B50" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C50" t="s">
         <v>2</v>
       </c>
       <c r="D50" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="E50" t="s">
-        <v>222</v>
+        <v>177</v>
       </c>
       <c r="F50" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="B51" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="C51" t="s">
         <v>8</v>
       </c>
       <c r="D51" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="E51" t="s">
-        <v>217</v>
+        <v>177</v>
       </c>
       <c r="F51" t="s">
-        <v>227</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" t="s">
-        <v>228</v>
+        <v>207</v>
       </c>
       <c r="B52" t="s">
-        <v>229</v>
+        <v>208</v>
       </c>
       <c r="C52" t="s">
         <v>8</v>
       </c>
       <c r="D52" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="E52" t="s">
-        <v>190</v>
+        <v>157</v>
       </c>
       <c r="F52" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
-        <v>230</v>
+        <v>209</v>
       </c>
       <c r="B53" t="s">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="C53" t="s">
         <v>2</v>
       </c>
       <c r="D53" t="s">
-        <v>232</v>
+        <v>211</v>
       </c>
       <c r="E53" t="s">
-        <v>233</v>
+        <v>157</v>
       </c>
       <c r="F53" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="B54" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="C54" t="s">
         <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="E54" t="s">
-        <v>238</v>
+        <v>157</v>
       </c>
       <c r="F54" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>239</v>
+        <v>216</v>
       </c>
       <c r="B55" t="s">
-        <v>240</v>
+        <v>217</v>
       </c>
       <c r="C55" t="s">
         <v>2</v>
       </c>
       <c r="D55" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="E55" t="s">
-        <v>242</v>
+        <v>219</v>
       </c>
       <c r="F55" t="s">
-        <v>243</v>
+        <v>220</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>244</v>
+        <v>221</v>
       </c>
       <c r="B56" t="s">
-        <v>245</v>
+        <v>222</v>
       </c>
       <c r="C56" t="s">
         <v>2</v>
       </c>
       <c r="D56" t="s">
-        <v>246</v>
+        <v>223</v>
       </c>
       <c r="E56" t="s">
-        <v>247</v>
+        <v>219</v>
       </c>
       <c r="F56" t="s">
-        <v>248</v>
+        <v>224</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
-        <v>249</v>
+        <v>225</v>
       </c>
       <c r="B57" t="s">
-        <v>250</v>
+        <v>226</v>
       </c>
       <c r="C57" t="s">
         <v>8</v>
       </c>
       <c r="D57" t="s">
-        <v>251</v>
+        <v>227</v>
       </c>
       <c r="E57" t="s">
-        <v>247</v>
+        <v>219</v>
       </c>
       <c r="F57" t="s">
-        <v>252</v>
+        <v>228</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>253</v>
+        <v>229</v>
       </c>
       <c r="B58" t="s">
-        <v>254</v>
+        <v>230</v>
       </c>
       <c r="C58" t="s">
         <v>2</v>
       </c>
       <c r="D58" t="s">
-        <v>255</v>
+        <v>231</v>
       </c>
       <c r="E58" t="s">
-        <v>256</v>
+        <v>232</v>
       </c>
       <c r="F58" t="s">
-        <v>257</v>
+        <v>233</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>258</v>
+        <v>234</v>
       </c>
       <c r="B59" t="s">
-        <v>259</v>
+        <v>235</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>260</v>
+        <v>236</v>
       </c>
       <c r="E59" t="s">
-        <v>261</v>
+        <v>232</v>
       </c>
       <c r="F59" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>263</v>
+        <v>238</v>
       </c>
       <c r="B60" t="s">
-        <v>264</v>
+        <v>239</v>
       </c>
       <c r="C60" t="s">
         <v>2</v>
       </c>
       <c r="D60" t="s">
-        <v>265</v>
+        <v>240</v>
       </c>
       <c r="E60" t="s">
-        <v>266</v>
+        <v>241</v>
       </c>
       <c r="F60" t="s">
-        <v>267</v>
+        <v>242</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>268</v>
+        <v>243</v>
       </c>
       <c r="B61" t="s">
-        <v>269</v>
+        <v>244</v>
       </c>
       <c r="C61" t="s">
         <v>2</v>
       </c>
       <c r="D61" t="s">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="E61" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F61" t="s">
-        <v>271</v>
+        <v>246</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>272</v>
+        <v>247</v>
       </c>
       <c r="B62" t="s">
-        <v>273</v>
+        <v>248</v>
       </c>
       <c r="C62" t="s">
         <v>8</v>
       </c>
       <c r="D62" t="s">
-        <v>274</v>
+        <v>249</v>
       </c>
       <c r="E62" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F62" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>275</v>
+        <v>250</v>
       </c>
       <c r="B63" t="s">
-        <v>276</v>
+        <v>251</v>
       </c>
       <c r="C63" t="s">
         <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>277</v>
+        <v>252</v>
       </c>
       <c r="E63" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F63" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>280</v>
+        <v>254</v>
       </c>
       <c r="B64" t="s">
-        <v>281</v>
+        <v>255</v>
       </c>
       <c r="C64" t="s">
         <v>2</v>
       </c>
       <c r="D64" t="s">
-        <v>282</v>
+        <v>256</v>
       </c>
       <c r="E64" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F64" t="s">
-        <v>283</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
-        <v>284</v>
+        <v>258</v>
       </c>
       <c r="B65" t="s">
-        <v>285</v>
+        <v>259</v>
       </c>
       <c r="C65" t="s">
         <v>8</v>
       </c>
       <c r="D65" t="s">
-        <v>286</v>
+        <v>260</v>
       </c>
       <c r="E65" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F65" t="s">
-        <v>287</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
-        <v>288</v>
+        <v>262</v>
       </c>
       <c r="B66" t="s">
-        <v>289</v>
+        <v>263</v>
       </c>
       <c r="C66" t="s">
         <v>8</v>
       </c>
       <c r="D66" t="s">
-        <v>290</v>
+        <v>264</v>
       </c>
       <c r="E66" t="s">
-        <v>222</v>
+        <v>177</v>
       </c>
       <c r="F66" t="s">
-        <v>291</v>
+        <v>265</v>
       </c>
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>292</v>
+        <v>266</v>
       </c>
       <c r="B67" t="s">
-        <v>293</v>
+        <v>267</v>
       </c>
       <c r="C67" t="s">
         <v>2</v>
       </c>
       <c r="D67" t="s">
-        <v>294</v>
+        <v>268</v>
       </c>
       <c r="E67" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="F67" t="s">
-        <v>295</v>
+        <v>269</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>296</v>
+        <v>270</v>
       </c>
       <c r="B68" t="s">
-        <v>293</v>
+        <v>267</v>
       </c>
       <c r="C68" t="s">
         <v>8</v>
       </c>
       <c r="D68" t="s">
-        <v>297</v>
+        <v>271</v>
       </c>
       <c r="E68" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="F68" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>298</v>
+        <v>272</v>
       </c>
       <c r="B69" t="s">
-        <v>299</v>
+        <v>273</v>
       </c>
       <c r="C69" t="s">
         <v>8</v>
       </c>
       <c r="D69" t="s">
-        <v>300</v>
+        <v>274</v>
       </c>
       <c r="E69" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F69" t="s">
-        <v>301</v>
+        <v>275</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" t="s">
-        <v>302</v>
+        <v>276</v>
       </c>
       <c r="B70" t="s">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="C70" t="s">
         <v>2</v>
       </c>
       <c r="D70" t="s">
-        <v>304</v>
+        <v>278</v>
       </c>
       <c r="E70" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F70" t="s">
-        <v>305</v>
+        <v>279</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" t="s">
-        <v>306</v>
+        <v>280</v>
       </c>
       <c r="B71" t="s">
-        <v>307</v>
+        <v>281</v>
       </c>
       <c r="C71" t="s">
         <v>2</v>
       </c>
       <c r="D71" t="s">
-        <v>308</v>
+        <v>282</v>
       </c>
       <c r="E71" t="s">
-        <v>309</v>
+        <v>283</v>
       </c>
       <c r="F71" t="s">
-        <v>310</v>
+        <v>284</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" t="s">
-        <v>311</v>
+        <v>285</v>
       </c>
       <c r="B72" t="s">
-        <v>312</v>
+        <v>286</v>
       </c>
       <c r="C72" t="s">
         <v>8</v>
       </c>
       <c r="D72" t="s">
-        <v>313</v>
+        <v>287</v>
       </c>
       <c r="E72" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="F72" t="s">
-        <v>314</v>
+        <v>288</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" t="s">
-        <v>315</v>
+        <v>289</v>
       </c>
       <c r="B73" t="s">
-        <v>316</v>
+        <v>290</v>
       </c>
       <c r="C73" t="s">
         <v>2</v>
       </c>
       <c r="D73" t="s">
-        <v>317</v>
+        <v>291</v>
       </c>
       <c r="E73" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F73" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
     </row>
     <row r="74" spans="1:6">
       <c r="A74" t="s">
-        <v>319</v>
+        <v>293</v>
       </c>
       <c r="B74" t="s">
-        <v>320</v>
+        <v>294</v>
       </c>
       <c r="C74" t="s">
         <v>8</v>
       </c>
       <c r="D74" t="s">
-        <v>321</v>
+        <v>295</v>
       </c>
       <c r="E74" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F74" t="s">
-        <v>322</v>
+        <v>296</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" t="s">
-        <v>323</v>
+        <v>297</v>
       </c>
       <c r="B75" t="s">
-        <v>324</v>
+        <v>298</v>
       </c>
       <c r="C75" t="s">
         <v>8</v>
       </c>
       <c r="D75" t="s">
-        <v>325</v>
+        <v>299</v>
       </c>
       <c r="E75" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F75" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="B76" t="s">
-        <v>328</v>
+        <v>302</v>
       </c>
       <c r="C76" t="s">
         <v>2</v>
       </c>
       <c r="D76" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="E76" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F76" t="s">
-        <v>330</v>
+        <v>304</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="B77" t="s">
-        <v>328</v>
+        <v>302</v>
       </c>
       <c r="C77" t="s">
         <v>8</v>
       </c>
       <c r="D77" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="E77" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F77" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
       <c r="B78" t="s">
-        <v>335</v>
+        <v>309</v>
       </c>
       <c r="C78" t="s">
         <v>2</v>
       </c>
       <c r="D78" t="s">
-        <v>336</v>
+        <v>310</v>
       </c>
       <c r="E78" t="s">
-        <v>337</v>
+        <v>311</v>
       </c>
       <c r="F78" t="s">
-        <v>338</v>
+        <v>312</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" t="s">
-        <v>339</v>
+        <v>313</v>
       </c>
       <c r="B79" t="s">
-        <v>340</v>
+        <v>314</v>
       </c>
       <c r="C79" t="s">
         <v>8</v>
       </c>
       <c r="D79" t="s">
-        <v>341</v>
+        <v>315</v>
       </c>
       <c r="E79" t="s">
-        <v>342</v>
+        <v>311</v>
       </c>
       <c r="F79" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" t="s">
-        <v>343</v>
+        <v>316</v>
       </c>
       <c r="B80" t="s">
-        <v>344</v>
+        <v>317</v>
       </c>
       <c r="C80" t="s">
         <v>2</v>
       </c>
       <c r="D80" t="s">
-        <v>345</v>
+        <v>318</v>
       </c>
       <c r="E80" t="s">
-        <v>346</v>
+        <v>319</v>
       </c>
       <c r="F80" t="s">
-        <v>347</v>
+        <v>320</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" t="s">
-        <v>348</v>
+        <v>321</v>
       </c>
       <c r="B81" t="s">
-        <v>349</v>
+        <v>322</v>
       </c>
       <c r="C81" t="s">
         <v>8</v>
       </c>
       <c r="D81" t="s">
-        <v>350</v>
+        <v>323</v>
       </c>
       <c r="E81" t="s">
-        <v>351</v>
+        <v>319</v>
       </c>
       <c r="F81" t="s">
-        <v>352</v>
+        <v>324</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="B82" t="s">
-        <v>354</v>
+        <v>326</v>
       </c>
       <c r="C82" t="s">
         <v>2</v>
       </c>
       <c r="D82" t="s">
-        <v>355</v>
+        <v>327</v>
       </c>
       <c r="E82" t="s">
-        <v>351</v>
+        <v>319</v>
       </c>
       <c r="F82" t="s">
-        <v>356</v>
+        <v>328</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="B83" t="s">
-        <v>358</v>
+        <v>330</v>
       </c>
       <c r="C83" t="s">
         <v>8</v>
       </c>
       <c r="D83" t="s">
-        <v>359</v>
+        <v>331</v>
       </c>
       <c r="E83" t="s">
-        <v>360</v>
+        <v>319</v>
       </c>
       <c r="F83" t="s">
-        <v>361</v>
+        <v>332</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="B84" t="s">
-        <v>363</v>
+        <v>334</v>
       </c>
       <c r="C84" t="s">
         <v>2</v>
       </c>
       <c r="D84" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
       <c r="E84" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F84" t="s">
-        <v>366</v>
+        <v>336</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" t="s">
-        <v>367</v>
+        <v>337</v>
       </c>
       <c r="B85" t="s">
-        <v>368</v>
+        <v>338</v>
       </c>
       <c r="C85" t="s">
         <v>2</v>
       </c>
       <c r="D85" t="s">
-        <v>369</v>
+        <v>339</v>
       </c>
       <c r="E85" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F85" t="s">
-        <v>370</v>
+        <v>340</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" t="s">
-        <v>371</v>
+        <v>341</v>
       </c>
       <c r="B86" t="s">
-        <v>372</v>
+        <v>342</v>
       </c>
       <c r="C86" t="s">
         <v>8</v>
       </c>
       <c r="D86" t="s">
-        <v>373</v>
+        <v>343</v>
       </c>
       <c r="E86" t="s">
-        <v>374</v>
+        <v>344</v>
       </c>
       <c r="F86" t="s">
-        <v>375</v>
+        <v>345</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" t="s">
-        <v>376</v>
+        <v>346</v>
       </c>
       <c r="B87" t="s">
-        <v>377</v>
+        <v>347</v>
       </c>
       <c r="C87" t="s">
         <v>2</v>
       </c>
       <c r="D87" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="E87" t="s">
-        <v>379</v>
+        <v>344</v>
       </c>
       <c r="F87" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" t="s">
-        <v>380</v>
+        <v>349</v>
       </c>
       <c r="B88" t="s">
-        <v>381</v>
+        <v>350</v>
       </c>
       <c r="C88" t="s">
         <v>8</v>
       </c>
       <c r="D88" t="s">
-        <v>382</v>
+        <v>351</v>
       </c>
       <c r="E88" t="s">
-        <v>383</v>
+        <v>352</v>
+      </c>
+      <c r="F88" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="B89" t="s">
-        <v>385</v>
+        <v>355</v>
       </c>
       <c r="C89" t="s">
         <v>2</v>
       </c>
       <c r="D89" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="E89" t="s">
-        <v>387</v>
+        <v>352</v>
       </c>
       <c r="F89" t="s">
-        <v>388</v>
+        <v>357</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" t="s">
-        <v>389</v>
+        <v>358</v>
       </c>
       <c r="B90" t="s">
-        <v>390</v>
+        <v>359</v>
       </c>
       <c r="C90" t="s">
         <v>2</v>
       </c>
       <c r="D90" t="s">
-        <v>391</v>
+        <v>360</v>
       </c>
       <c r="E90" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F90" t="s">
-        <v>392</v>
+        <v>361</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" t="s">
-        <v>393</v>
+        <v>362</v>
       </c>
       <c r="B91" t="s">
-        <v>394</v>
+        <v>363</v>
       </c>
       <c r="C91" t="s">
         <v>2</v>
       </c>
       <c r="D91" t="s">
-        <v>395</v>
+        <v>364</v>
       </c>
       <c r="E91" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F91" t="s">
-        <v>396</v>
+        <v>365</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" t="s">
-        <v>397</v>
+        <v>366</v>
       </c>
       <c r="B92" t="s">
-        <v>394</v>
+        <v>363</v>
       </c>
       <c r="C92" t="s">
         <v>8</v>
       </c>
       <c r="D92" t="s">
-        <v>398</v>
+        <v>367</v>
       </c>
       <c r="E92" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F92" t="s">
-        <v>399</v>
+        <v>368</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" t="s">
-        <v>400</v>
+        <v>369</v>
       </c>
       <c r="B93" t="s">
-        <v>401</v>
+        <v>370</v>
       </c>
       <c r="C93" t="s">
         <v>8</v>
       </c>
       <c r="D93" t="s">
-        <v>402</v>
+        <v>371</v>
       </c>
       <c r="E93" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F93" t="s">
-        <v>403</v>
+        <v>372</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" t="s">
-        <v>404</v>
+        <v>373</v>
       </c>
       <c r="B94" t="s">
-        <v>405</v>
+        <v>374</v>
       </c>
       <c r="C94" t="s">
         <v>2</v>
       </c>
       <c r="D94" t="s">
-        <v>406</v>
+        <v>375</v>
       </c>
       <c r="E94" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F94" t="s">
-        <v>407</v>
+        <v>376</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" t="s">
-        <v>408</v>
+        <v>377</v>
       </c>
       <c r="B95" t="s">
-        <v>409</v>
+        <v>378</v>
       </c>
       <c r="C95" t="s">
         <v>8</v>
       </c>
       <c r="D95" t="s">
-        <v>410</v>
+        <v>379</v>
       </c>
       <c r="E95" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="F95" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" t="s">
-        <v>411</v>
+        <v>380</v>
       </c>
       <c r="B96" t="s">
-        <v>412</v>
+        <v>381</v>
       </c>
       <c r="C96" t="s">
         <v>2</v>
       </c>
       <c r="D96" t="s">
-        <v>413</v>
+        <v>382</v>
       </c>
       <c r="E96" t="s">
-        <v>414</v>
+        <v>383</v>
       </c>
       <c r="F96" t="s">
-        <v>415</v>
+        <v>384</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" t="s">
-        <v>416</v>
+        <v>385</v>
       </c>
       <c r="B97" t="s">
-        <v>417</v>
+        <v>386</v>
       </c>
       <c r="C97" t="s">
         <v>8</v>
       </c>
       <c r="D97" t="s">
-        <v>418</v>
+        <v>387</v>
       </c>
       <c r="E97" t="s">
-        <v>419</v>
+        <v>383</v>
       </c>
       <c r="F97" t="s">
-        <v>420</v>
+        <v>388</v>
       </c>
     </row>
     <row r="98" spans="1:6">
       <c r="A98" t="s">
-        <v>421</v>
+        <v>389</v>
       </c>
       <c r="B98" t="s">
-        <v>422</v>
+        <v>390</v>
       </c>
       <c r="C98" t="s">
         <v>2</v>
       </c>
       <c r="D98" t="s">
-        <v>423</v>
+        <v>391</v>
       </c>
       <c r="E98" t="s">
-        <v>424</v>
+        <v>392</v>
       </c>
       <c r="F98" t="s">
-        <v>425</v>
+        <v>393</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" t="s">
-        <v>426</v>
+        <v>394</v>
       </c>
       <c r="B99" t="s">
-        <v>427</v>
+        <v>395</v>
       </c>
       <c r="C99" t="s">
         <v>8</v>
       </c>
       <c r="D99" t="s">
-        <v>428</v>
+        <v>396</v>
       </c>
       <c r="E99" t="s">
-        <v>429</v>
+        <v>397</v>
       </c>
       <c r="F99" t="s">
-        <v>430</v>
+        <v>398</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" t="s">
-        <v>431</v>
+        <v>399</v>
       </c>
       <c r="B100" t="s">
-        <v>432</v>
+        <v>400</v>
       </c>
       <c r="C100" t="s">
         <v>2</v>
       </c>
       <c r="D100" t="s">
-        <v>433</v>
+        <v>401</v>
       </c>
       <c r="E100" t="s">
-        <v>434</v>
+        <v>397</v>
       </c>
       <c r="F100" t="s">
-        <v>435</v>
+        <v>402</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" t="s">
-        <v>436</v>
+        <v>403</v>
       </c>
       <c r="B101" t="s">
-        <v>437</v>
+        <v>404</v>
       </c>
       <c r="C101" t="s">
         <v>8</v>
       </c>
       <c r="D101" t="s">
-        <v>438</v>
+        <v>405</v>
       </c>
       <c r="E101" t="s">
-        <v>439</v>
+        <v>406</v>
       </c>
       <c r="F101" t="s">
-        <v>440</v>
+        <v>407</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" t="s">
-        <v>441</v>
+        <v>408</v>
       </c>
       <c r="B102" t="s">
-        <v>442</v>
+        <v>409</v>
       </c>
       <c r="C102" t="s">
         <v>2</v>
       </c>
       <c r="D102" t="s">
-        <v>443</v>
+        <v>410</v>
       </c>
       <c r="E102" t="s">
-        <v>444</v>
+        <v>406</v>
       </c>
       <c r="F102" t="s">
-        <v>445</v>
+        <v>411</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" t="s">
-        <v>446</v>
+        <v>412</v>
       </c>
       <c r="B103" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C103" t="s">
         <v>2</v>
       </c>
       <c r="D103" t="s">
-        <v>448</v>
+        <v>414</v>
       </c>
       <c r="E103" t="s">
-        <v>449</v>
+        <v>415</v>
       </c>
       <c r="F103" t="s">
-        <v>450</v>
+        <v>416</v>
       </c>
     </row>
     <row r="104" spans="1:6">
       <c r="A104" t="s">
-        <v>451</v>
+        <v>417</v>
       </c>
       <c r="B104" t="s">
-        <v>452</v>
+        <v>418</v>
       </c>
       <c r="C104" t="s">
         <v>8</v>
       </c>
       <c r="D104" t="s">
-        <v>453</v>
+        <v>419</v>
       </c>
       <c r="E104" t="s">
-        <v>454</v>
+        <v>415</v>
       </c>
       <c r="F104" t="s">
-        <v>455</v>
+        <v>420</v>
       </c>
     </row>
     <row r="105" spans="1:6">
       <c r="A105" t="s">
-        <v>456</v>
+        <v>421</v>
       </c>
       <c r="B105" t="s">
-        <v>457</v>
+        <v>422</v>
       </c>
       <c r="C105" t="s">
         <v>2</v>
       </c>
       <c r="D105" t="s">
-        <v>458</v>
+        <v>423</v>
       </c>
       <c r="E105" t="s">
-        <v>454</v>
+        <v>415</v>
       </c>
       <c r="F105" t="s">
-        <v>459</v>
+        <v>424</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" t="s">
-        <v>460</v>
+        <v>425</v>
       </c>
       <c r="B106" t="s">
-        <v>461</v>
+        <v>426</v>
       </c>
       <c r="C106" t="s">
         <v>8</v>
       </c>
       <c r="D106" t="s">
-        <v>462</v>
+        <v>427</v>
       </c>
       <c r="E106" t="s">
-        <v>454</v>
+        <v>415</v>
       </c>
       <c r="F106" t="s">
-        <v>463</v>
+        <v>428</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" t="s">
-        <v>464</v>
+        <v>429</v>
       </c>
       <c r="B107" t="s">
-        <v>465</v>
+        <v>430</v>
       </c>
       <c r="C107" t="s">
         <v>8</v>
       </c>
       <c r="D107" t="s">
-        <v>466</v>
+        <v>431</v>
       </c>
       <c r="E107" t="s">
-        <v>467</v>
+        <v>432</v>
       </c>
       <c r="F107" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" t="s">
-        <v>468</v>
+        <v>433</v>
       </c>
       <c r="B108" t="s">
-        <v>469</v>
+        <v>434</v>
       </c>
       <c r="C108" t="s">
         <v>8</v>
       </c>
       <c r="D108" t="s">
-        <v>466</v>
+        <v>431</v>
       </c>
       <c r="E108" t="s">
-        <v>470</v>
+        <v>435</v>
       </c>
       <c r="F108" t="s">
-        <v>471</v>
+        <v>436</v>
       </c>
     </row>
     <row r="109" spans="1:6">
       <c r="A109" t="s">
-        <v>472</v>
+        <v>437</v>
       </c>
       <c r="B109" t="s">
-        <v>473</v>
+        <v>438</v>
       </c>
       <c r="C109" t="s">
         <v>2</v>
       </c>
       <c r="D109" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="E109" t="s">
-        <v>475</v>
+        <v>432</v>
       </c>
       <c r="F109" t="s">
-        <v>476</v>
+        <v>440</v>
       </c>
     </row>
     <row r="110" spans="1:6">
       <c r="A110" t="s">
-        <v>477</v>
+        <v>441</v>
       </c>
       <c r="B110" t="s">
-        <v>478</v>
+        <v>442</v>
       </c>
       <c r="C110" t="s">
         <v>2</v>
       </c>
       <c r="D110" t="s">
-        <v>479</v>
+        <v>443</v>
       </c>
       <c r="E110" t="s">
-        <v>480</v>
+        <v>435</v>
       </c>
       <c r="F110" t="s">
-        <v>481</v>
+        <v>444</v>
       </c>
     </row>
     <row r="111" spans="1:6">
       <c r="A111" t="s">
-        <v>482</v>
+        <v>445</v>
       </c>
       <c r="B111" t="s">
-        <v>483</v>
+        <v>446</v>
       </c>
       <c r="C111" t="s">
         <v>8</v>
       </c>
       <c r="D111" t="s">
-        <v>484</v>
+        <v>447</v>
       </c>
       <c r="E111" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F111" t="s">
-        <v>485</v>
+        <v>448</v>
       </c>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" t="s">
-        <v>486</v>
+        <v>449</v>
       </c>
       <c r="B112" t="s">
-        <v>487</v>
+        <v>450</v>
       </c>
       <c r="C112" t="s">
         <v>2</v>
       </c>
       <c r="D112" t="s">
-        <v>488</v>
+        <v>451</v>
       </c>
       <c r="E112" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F112" t="s">
-        <v>489</v>
+        <v>452</v>
       </c>
     </row>
     <row r="113" spans="1:6">
       <c r="A113" t="s">
-        <v>490</v>
+        <v>453</v>
       </c>
       <c r="B113" t="s">
-        <v>491</v>
+        <v>454</v>
       </c>
       <c r="C113" t="s">
         <v>8</v>
       </c>
       <c r="D113" t="s">
-        <v>492</v>
+        <v>455</v>
       </c>
       <c r="E113" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F113" t="s">
-        <v>493</v>
+        <v>456</v>
       </c>
     </row>
     <row r="114" spans="1:6">
       <c r="A114" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="B114" t="s">
-        <v>495</v>
+        <v>458</v>
       </c>
       <c r="C114" t="s">
         <v>8</v>
       </c>
       <c r="D114" t="s">
-        <v>496</v>
+        <v>459</v>
       </c>
       <c r="E114" t="s">
-        <v>497</v>
+        <v>460</v>
       </c>
       <c r="F114" t="s">
-        <v>498</v>
+        <v>461</v>
       </c>
     </row>
     <row r="115" spans="1:6">
       <c r="A115" t="s">
-        <v>499</v>
+        <v>462</v>
       </c>
       <c r="B115" t="s">
-        <v>500</v>
+        <v>463</v>
       </c>
       <c r="C115" t="s">
         <v>8</v>
       </c>
       <c r="D115" t="s">
-        <v>496</v>
+        <v>459</v>
       </c>
       <c r="E115" t="s">
-        <v>501</v>
+        <v>464</v>
       </c>
       <c r="F115" t="s">
-        <v>502</v>
+        <v>465</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" t="s">
-        <v>503</v>
+        <v>466</v>
       </c>
       <c r="B116" t="s">
-        <v>504</v>
+        <v>467</v>
       </c>
       <c r="C116" t="s">
         <v>2</v>
       </c>
       <c r="D116" t="s">
-        <v>505</v>
+        <v>468</v>
       </c>
       <c r="E116" t="s">
-        <v>506</v>
+        <v>464</v>
       </c>
       <c r="F116" t="s">
-        <v>507</v>
+        <v>469</v>
       </c>
     </row>
     <row r="117" spans="1:6">
       <c r="A117" t="s">
-        <v>508</v>
+        <v>470</v>
       </c>
       <c r="B117" t="s">
-        <v>509</v>
+        <v>471</v>
       </c>
       <c r="C117" t="s">
         <v>2</v>
       </c>
       <c r="D117" t="s">
-        <v>510</v>
+        <v>472</v>
       </c>
       <c r="E117" t="s">
-        <v>511</v>
+        <v>460</v>
       </c>
       <c r="F117" t="s">
-        <v>512</v>
+        <v>473</v>
       </c>
     </row>
     <row r="118" spans="1:6">
       <c r="A118" t="s">
-        <v>513</v>
+        <v>474</v>
       </c>
       <c r="B118" t="s">
-        <v>509</v>
+        <v>471</v>
       </c>
       <c r="C118" t="s">
         <v>2</v>
       </c>
       <c r="D118" t="s">
-        <v>510</v>
+        <v>472</v>
       </c>
       <c r="E118" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="F118" t="s">
-        <v>514</v>
+        <v>475</v>
       </c>
     </row>
     <row r="119" spans="1:6">
       <c r="A119" t="s">
-        <v>515</v>
+        <v>476</v>
       </c>
       <c r="B119" t="s">
-        <v>516</v>
+        <v>477</v>
       </c>
       <c r="C119" t="s">
         <v>8</v>
       </c>
       <c r="D119" t="s">
-        <v>517</v>
+        <v>478</v>
       </c>
       <c r="E119" t="s">
-        <v>511</v>
+        <v>460</v>
       </c>
       <c r="F119" t="s">
-        <v>518</v>
+        <v>479</v>
       </c>
     </row>
     <row r="120" spans="1:6">
       <c r="A120" t="s">
-        <v>519</v>
+        <v>480</v>
       </c>
       <c r="B120" t="s">
-        <v>520</v>
+        <v>481</v>
       </c>
       <c r="C120" t="s">
         <v>2</v>
       </c>
       <c r="D120" t="s">
-        <v>521</v>
+        <v>482</v>
       </c>
       <c r="E120" t="s">
-        <v>511</v>
+        <v>460</v>
       </c>
       <c r="F120" t="s">
-        <v>522</v>
+        <v>483</v>
       </c>
     </row>
     <row r="121" spans="1:6">
       <c r="A121" t="s">
-        <v>523</v>
+        <v>484</v>
       </c>
       <c r="B121" t="s">
-        <v>524</v>
+        <v>485</v>
       </c>
       <c r="C121" t="s">
         <v>8</v>
       </c>
       <c r="D121" t="s">
-        <v>525</v>
+        <v>486</v>
       </c>
       <c r="E121" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="F121" t="s">
-        <v>527</v>
+        <v>488</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" t="s">
-        <v>528</v>
+        <v>489</v>
       </c>
       <c r="B122" t="s">
-        <v>529</v>
+        <v>490</v>
       </c>
       <c r="C122" t="s">
         <v>2</v>
       </c>
       <c r="D122" t="s">
-        <v>530</v>
+        <v>491</v>
       </c>
       <c r="E122" t="s">
-        <v>531</v>
+        <v>487</v>
       </c>
       <c r="F122" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
     </row>
     <row r="123" spans="1:6">
       <c r="A123" t="s">
-        <v>532</v>
+        <v>492</v>
       </c>
       <c r="B123" t="s">
-        <v>533</v>
+        <v>493</v>
       </c>
       <c r="C123" t="s">
         <v>2</v>
       </c>
       <c r="D123" t="s">
-        <v>534</v>
+        <v>494</v>
       </c>
       <c r="E123" t="s">
-        <v>535</v>
+        <v>495</v>
       </c>
       <c r="F123" t="s">
-        <v>536</v>
+        <v>496</v>
       </c>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" t="s">
-        <v>537</v>
+        <v>497</v>
       </c>
       <c r="B124" t="s">
-        <v>538</v>
+        <v>498</v>
       </c>
       <c r="C124" t="s">
         <v>2</v>
       </c>
       <c r="D124" t="s">
-        <v>539</v>
+        <v>499</v>
       </c>
       <c r="E124" t="s">
-        <v>540</v>
+        <v>500</v>
       </c>
       <c r="F124" t="s">
-        <v>541</v>
+        <v>501</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" t="s">
-        <v>542</v>
+        <v>502</v>
       </c>
       <c r="B125" t="s">
-        <v>543</v>
+        <v>503</v>
       </c>
       <c r="C125" t="s">
         <v>8</v>
       </c>
       <c r="D125" t="s">
-        <v>544</v>
+        <v>504</v>
       </c>
       <c r="E125" t="s">
-        <v>545</v>
+        <v>495</v>
       </c>
       <c r="F125" t="s">
-        <v>546</v>
+        <v>505</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" t="s">
-        <v>547</v>
+        <v>506</v>
       </c>
       <c r="B126" t="s">
-        <v>548</v>
+        <v>507</v>
       </c>
       <c r="C126" t="s">
         <v>2</v>
       </c>
       <c r="D126" t="s">
-        <v>549</v>
+        <v>508</v>
       </c>
       <c r="E126" t="s">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="F126" t="s">
-        <v>551</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>